<commit_message>
Added Freelance project tracker and srms
</commit_message>
<xml_diff>
--- a/Simple-Projects/excel-report-generator/sales_report.xlsx
+++ b/Simple-Projects/excel-report-generator/sales_report.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cleaned Data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary by SalesPerson" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Summary by Region" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cleaned Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary by SalesPerson" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Best Product by Region" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overall Summary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -432,13 +433,13 @@
   <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="7" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -957,10 +958,10 @@
   <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1143,9 +1144,9 @@
   <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1156,7 +1157,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Best_Product</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -1238,6 +1239,114 @@
       </c>
       <c r="C6" t="n">
         <v>1575</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Total Revenue</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>£14,874.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Total Units Sold</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>730.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Total Orders</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Average Order Value</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>£991.62</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Number of Sales Persons</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Number of Regions</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Number of Products</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>